<commit_message>
Deploying to gh-pages from  @ 62c0fa2b2b7de82e179b578871239bb279a9d53c 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_1-1-1.xlsx
+++ b/assets/excel/2026_1-1-1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89BB305-7255-416A-9813-BDBB32F01A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74EE4D1A-E4B7-44B1-A142-40B08BAD5F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{10A5E901-1E3B-4FD8-A95C-5E70FBB58270}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{10A5E901-1E3B-4FD8-A95C-5E70FBB58270}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
   <si>
     <t>Kreisfreie Stadt
 Landkreis
@@ -258,6 +258,9 @@
   </si>
   <si>
     <t>Quelle: Bevölkerungsfortschreibung</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -539,9 +542,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -579,7 +582,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -685,7 +688,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -827,7 +830,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -836,7 +839,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{017B5BDD-0A11-45EA-8564-DA0C056DBCB1}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="B1:AA72"/>
+  <dimension ref="A1:AA72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
@@ -844,23 +847,29 @@
     <col min="3" max="3" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
       <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="19" t="s">
         <v>0</v>
       </c>
@@ -893,7 +902,7 @@
       <c r="Z7" s="23"/>
       <c r="AA7" s="23"/>
     </row>
-    <row r="8" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="C8" s="20"/>
       <c r="D8" s="13">
         <v>2005</v>
@@ -968,7 +977,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="C9" s="21"/>
       <c r="D9" s="22" t="s">
         <v>3</v>
@@ -999,7 +1008,7 @@
       <c r="Z9" s="23"/>
       <c r="AA9" s="23"/>
     </row>
-    <row r="10" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="C10" s="16">
         <v>1</v>
       </c>
@@ -1076,7 +1085,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="2:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <v>101</v>
       </c>
@@ -1156,7 +1165,7 @@
         <v>-5.9728413716175321E-2</v>
       </c>
     </row>
-    <row r="12" spans="2:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <v>102</v>
       </c>
@@ -1236,7 +1245,7 @@
         <v>-0.51420527994024878</v>
       </c>
     </row>
-    <row r="13" spans="2:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <v>103</v>
       </c>
@@ -1316,7 +1325,7 @@
         <v>0.19489573463366536</v>
       </c>
     </row>
-    <row r="14" spans="2:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <v>151</v>
       </c>
@@ -1396,7 +1405,7 @@
         <v>-0.2421404072516779</v>
       </c>
     </row>
-    <row r="15" spans="2:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <v>153</v>
       </c>
@@ -1476,7 +1485,7 @@
         <v>-0.54964229628337113</v>
       </c>
     </row>
-    <row r="16" spans="2:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" s="3" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <v>154</v>
       </c>

</xml_diff>